<commit_message>
Actualizar DOMMA_Analisis_Menopausia_BA.xlsx - 30/03/2026 16:39
</commit_message>
<xml_diff>
--- a/DOMMA_Analisis_Menopausia_BA.xlsx
+++ b/DOMMA_Analisis_Menopausia_BA.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>79640</v>
+        <v>88162</v>
       </c>
     </row>
     <row r="3">
@@ -500,7 +500,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>30/03/2026 16:37</t>
+          <t>30/03/2026 16:39</t>
         </is>
       </c>
     </row>
@@ -584,6 +584,16 @@
         <is>
           <t>2025-08-26</t>
         </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Nuevo: DOMMA_Quiz_responses_2026-03-30_142714.csv</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>8522</v>
       </c>
     </row>
   </sheetData>
@@ -622,7 +632,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>74.5</v>
+        <v>67.3</v>
       </c>
     </row>
     <row r="3">
@@ -632,7 +642,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>64.59999999999999</v>
+        <v>58.3</v>
       </c>
     </row>
     <row r="4">
@@ -642,7 +652,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>63.6</v>
+        <v>57.4</v>
       </c>
     </row>
     <row r="5">
@@ -652,7 +662,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>63.1</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6">
@@ -662,7 +672,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>57.1</v>
+        <v>51.6</v>
       </c>
     </row>
     <row r="7">
@@ -672,7 +682,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>56.5</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8">
@@ -682,7 +692,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>53</v>
+        <v>47.9</v>
       </c>
     </row>
     <row r="9">
@@ -692,7 +702,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>43</v>
+        <v>38.8</v>
       </c>
     </row>
     <row r="10">
@@ -702,7 +712,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>41.7</v>
+        <v>37.6</v>
       </c>
     </row>
     <row r="11">
@@ -712,7 +722,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>38.4</v>
+        <v>34.7</v>
       </c>
     </row>
   </sheetData>
@@ -751,7 +761,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>45.2</v>
+        <v>40.8</v>
       </c>
     </row>
     <row r="3">
@@ -761,7 +771,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>41.5</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="4">
@@ -771,7 +781,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>38.5</v>
+        <v>34.8</v>
       </c>
     </row>
     <row r="5">
@@ -781,7 +791,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>37.4</v>
+        <v>33.8</v>
       </c>
     </row>
     <row r="6">
@@ -791,7 +801,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>36.9</v>
+        <v>33.4</v>
       </c>
     </row>
     <row r="7">
@@ -801,7 +811,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>36.7</v>
+        <v>33.2</v>
       </c>
     </row>
     <row r="8">
@@ -811,7 +821,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2.4</v>
+        <v>2.2</v>
       </c>
     </row>
   </sheetData>
@@ -855,10 +865,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>33216</v>
+        <v>37693</v>
       </c>
       <c r="C2" t="n">
-        <v>41.7</v>
+        <v>42.8</v>
       </c>
     </row>
     <row r="3">
@@ -868,10 +878,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>23226</v>
+        <v>25006</v>
       </c>
       <c r="C3" t="n">
-        <v>29.2</v>
+        <v>28.4</v>
       </c>
     </row>
     <row r="4">
@@ -881,10 +891,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>14051</v>
+        <v>15381</v>
       </c>
       <c r="C4" t="n">
-        <v>17.6</v>
+        <v>17.4</v>
       </c>
     </row>
     <row r="5">
@@ -894,10 +904,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6603</v>
+        <v>7538</v>
       </c>
       <c r="C5" t="n">
-        <v>8.300000000000001</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="6">
@@ -910,7 +920,7 @@
         <v>1850</v>
       </c>
       <c r="C6" t="n">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="7">
@@ -949,7 +959,7 @@
         <v>124</v>
       </c>
       <c r="C9" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="10">
@@ -1001,7 +1011,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>83.3</v>
+        <v>84.40000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -1011,7 +1021,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10.7</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="4">
@@ -1021,7 +1031,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3.1</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="5">
@@ -1031,7 +1041,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="6">

</xml_diff>